<commit_message>
email, mượn trả sách
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/Import1.xlsx
+++ b/src/main/resources/templates/Import1.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="13128" windowHeight="4392"/>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="48">
   <si>
     <t>STT</t>
   </si>
@@ -35,13 +35,16 @@
     <t>Mã thành viên</t>
   </si>
   <si>
+    <t>Cccd</t>
+  </si>
+  <si>
     <t>Tên thành viên</t>
   </si>
   <si>
     <t>Email</t>
   </si>
   <si>
-    <t>SĐT</t>
+    <t>Số điện thoại</t>
   </si>
   <si>
     <t>Trạng thái</t>
@@ -50,97 +53,124 @@
     <t>Mô tả</t>
   </si>
   <si>
-    <t>M1</t>
-  </si>
-  <si>
-    <t>Ba lăng nhằng</t>
-  </si>
-  <si>
-    <t>aaa4</t>
-  </si>
-  <si>
-    <t>Đây là thành viên</t>
-  </si>
-  <si>
-    <t>M2</t>
-  </si>
-  <si>
-    <t>nva@gmail.com</t>
-  </si>
-  <si>
-    <t>0323456789</t>
-  </si>
-  <si>
-    <t>M3</t>
-  </si>
-  <si>
-    <t>nvb@gmail.com</t>
-  </si>
-  <si>
-    <t>0323456790</t>
-  </si>
-  <si>
-    <t>M4</t>
-  </si>
-  <si>
-    <t>nvc@gmail.com</t>
-  </si>
-  <si>
-    <t>0323456791</t>
-  </si>
-  <si>
-    <t>M5</t>
-  </si>
-  <si>
-    <t>nvd@gmail.com</t>
-  </si>
-  <si>
-    <t>0323456792</t>
-  </si>
-  <si>
-    <t>M6</t>
-  </si>
-  <si>
-    <t>nve@gmail.com</t>
-  </si>
-  <si>
-    <t>0323456793</t>
-  </si>
-  <si>
-    <t>M7</t>
-  </si>
-  <si>
-    <t>nvf@gmail.com</t>
-  </si>
-  <si>
-    <t>0323456794</t>
-  </si>
-  <si>
-    <t>M8</t>
-  </si>
-  <si>
-    <t>nvg@gmail.com</t>
-  </si>
-  <si>
-    <t>0323456795</t>
-  </si>
-  <si>
-    <t>M9</t>
-  </si>
-  <si>
-    <t>nvh@gmail.com</t>
-  </si>
-  <si>
-    <t>0323456796</t>
-  </si>
-  <si>
-    <t>M10</t>
-  </si>
-  <si>
-    <t>nvj@gmail.com</t>
-  </si>
-  <si>
-    <t>0323456797</t>
+    <t>KK1</t>
+  </si>
+  <si>
+    <t>098123456789</t>
+  </si>
+  <si>
+    <t>Nạp cô cô</t>
+  </si>
+  <si>
+    <t>Thành viên</t>
+  </si>
+  <si>
+    <t>KK2</t>
+  </si>
+  <si>
+    <t>097123456789</t>
+  </si>
+  <si>
+    <t>cct12@gmail.com</t>
+  </si>
+  <si>
+    <t>0922345678</t>
+  </si>
+  <si>
+    <t>KK3</t>
+  </si>
+  <si>
+    <t>096123456789</t>
+  </si>
+  <si>
+    <t>cct13@gmail.com</t>
+  </si>
+  <si>
+    <t>0925345679</t>
+  </si>
+  <si>
+    <t>KK4</t>
+  </si>
+  <si>
+    <t>095123456789</t>
+  </si>
+  <si>
+    <t>cct14@gmail.com</t>
+  </si>
+  <si>
+    <t>0926345680</t>
+  </si>
+  <si>
+    <t>KK5</t>
+  </si>
+  <si>
+    <t>094123456789</t>
+  </si>
+  <si>
+    <t>cct15@gmail.com</t>
+  </si>
+  <si>
+    <t>0952345681</t>
+  </si>
+  <si>
+    <t>KK6</t>
+  </si>
+  <si>
+    <t>093123456789</t>
+  </si>
+  <si>
+    <t>cct16@gmail.com</t>
+  </si>
+  <si>
+    <t>0928345682</t>
+  </si>
+  <si>
+    <t>KK7</t>
+  </si>
+  <si>
+    <t>092123456789</t>
+  </si>
+  <si>
+    <t>cct17@gmail.com</t>
+  </si>
+  <si>
+    <t>0942345683</t>
+  </si>
+  <si>
+    <t>KK8</t>
+  </si>
+  <si>
+    <t>091123456789</t>
+  </si>
+  <si>
+    <t>cct18@gmail.com</t>
+  </si>
+  <si>
+    <t>0992345684</t>
+  </si>
+  <si>
+    <t>KK9</t>
+  </si>
+  <si>
+    <t>090123456789</t>
+  </si>
+  <si>
+    <t>cct19@gmail.com</t>
+  </si>
+  <si>
+    <t>0999345685</t>
+  </si>
+  <si>
+    <t>KK10</t>
+  </si>
+  <si>
+    <t>091023456789</t>
+  </si>
+  <si>
+    <t>cct20@gmail.com</t>
+  </si>
+  <si>
+    <t>0922399686</t>
   </si>
 </sst>
 </file>
@@ -1294,18 +1324,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="6"/>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
     <col min="2" max="2" width="12.6666666666667" customWidth="1"/>
     <col min="3" max="3" width="14.7777777777778" customWidth="1"/>
     <col min="4" max="4" width="17.7777777777778" customWidth="1"/>
-    <col min="5" max="5" width="13.3333333333333" customWidth="1"/>
-    <col min="6" max="6" width="10.4444444444444" customWidth="1"/>
+    <col min="5" max="5" width="18.5555555555556" customWidth="1"/>
+    <col min="6" max="6" width="13.2222222222222" customWidth="1"/>
     <col min="7" max="7" width="16.2222222222222" customWidth="1"/>
+    <col min="8" max="8" width="15.5555555555556" customWidth="1"/>
+    <col min="9" max="9" width="22.6666666666667" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1327,248 +1359,281 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:8">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
         <v>8</v>
       </c>
+      <c r="C2" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="D2" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E2">
         <v>50.4</v>
       </c>
-      <c r="F2" t="b">
+      <c r="F2">
+        <v>25</v>
+      </c>
+      <c r="G2" t="b">
         <v>1</v>
       </c>
-      <c r="G2" t="s">
-        <v>10</v>
+      <c r="H2" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:8">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G3" t="s">
-        <v>10</v>
-      </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:8">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F4" t="b">
+      <c r="C4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" t="b">
         <v>1</v>
       </c>
-      <c r="G4" t="s">
-        <v>10</v>
+      <c r="H4" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:8">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" t="b">
+        <v>10</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" t="b">
         <v>1</v>
       </c>
-      <c r="G5" t="s">
-        <v>10</v>
+      <c r="H5" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:8">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" t="b">
+        <v>24</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" t="b">
         <v>1</v>
       </c>
-      <c r="G6" t="s">
-        <v>10</v>
+      <c r="H6" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:8">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" t="b">
+        <v>28</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" t="b">
         <v>1</v>
       </c>
-      <c r="G7" t="s">
-        <v>10</v>
+      <c r="H7" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:8">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F8" t="b">
+        <v>32</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G8" t="b">
         <v>1</v>
       </c>
-      <c r="G8" t="s">
-        <v>10</v>
+      <c r="H8" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:8">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
-      </c>
-      <c r="C9" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="F9" t="b">
+        <v>36</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G9" t="b">
         <v>1</v>
       </c>
-      <c r="G9" t="s">
-        <v>10</v>
+      <c r="H9" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:8">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F10" t="b">
+        <v>40</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="G10" t="b">
         <v>1</v>
       </c>
-      <c r="G10" t="s">
-        <v>10</v>
+      <c r="H10" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:8">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F11" t="b">
+        <v>44</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="G11" t="b">
         <v>1</v>
       </c>
-      <c r="G11" t="s">
-        <v>10</v>
+      <c r="H11" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D3" r:id="rId1" display="nva@gmail.com"/>
-    <hyperlink ref="D4" r:id="rId2" display="nvb@gmail.com"/>
-    <hyperlink ref="D5" r:id="rId3" display="nvc@gmail.com" tooltip="mailto:nvc@gmail.com"/>
-    <hyperlink ref="D6" r:id="rId4" display="nvd@gmail.com" tooltip="mailto:nvd@gmail.com"/>
-    <hyperlink ref="D7" r:id="rId5" display="nve@gmail.com" tooltip="mailto:nve@gmail.com"/>
-    <hyperlink ref="D8" r:id="rId6" display="nvf@gmail.com" tooltip="mailto:nvf@gmail.com"/>
-    <hyperlink ref="D9" r:id="rId7" display="nvg@gmail.com" tooltip="mailto:nvg@gmail.com"/>
-    <hyperlink ref="D10" r:id="rId8" display="nvh@gmail.com" tooltip="mailto:nvh@gmail.com"/>
-    <hyperlink ref="D11" r:id="rId9" display="nvj@gmail.com" tooltip="mailto:nvj@gmail.com"/>
+    <hyperlink ref="E3" r:id="rId1" display="cct12@gmail.com" tooltip="mailto:cct12@gmail.com"/>
+    <hyperlink ref="E4" r:id="rId1" display="cct13@gmail.com" tooltip="mailto:cct12@gmail.com"/>
+    <hyperlink ref="E5" r:id="rId1" display="cct14@gmail.com" tooltip="mailto:cct12@gmail.com"/>
+    <hyperlink ref="E6" r:id="rId1" display="cct15@gmail.com" tooltip="mailto:cct12@gmail.com"/>
+    <hyperlink ref="E7" r:id="rId1" display="cct16@gmail.com" tooltip="mailto:cct12@gmail.com"/>
+    <hyperlink ref="E8" r:id="rId1" display="cct17@gmail.com" tooltip="mailto:cct12@gmail.com"/>
+    <hyperlink ref="E9" r:id="rId1" display="cct18@gmail.com" tooltip="mailto:cct12@gmail.com"/>
+    <hyperlink ref="E10" r:id="rId1" display="cct19@gmail.com" tooltip="mailto:cct12@gmail.com"/>
+    <hyperlink ref="E11" r:id="rId1" display="cct20@gmail.com" tooltip="mailto:cct12@gmail.com"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>